<commit_message>
Random Forest Feature Engeneering script
</commit_message>
<xml_diff>
--- a/RandomForest_Outputs/agriculture_cereal_best_random_forest_results.xlsx
+++ b/RandomForest_Outputs/agriculture_cereal_best_random_forest_results.xlsx
@@ -5,16 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eskom-my.sharepoint.com/personal/mauduh_eskom_co_za/Documents/Python Projects/Parameter-Optimisation/RandomForest_Search_Outputs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eskom-my.sharepoint.com/personal/mauduh_eskom_co_za/Documents/Python Projects/Parameter-Optimisation/RandomForest_Outputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_2B59D2BFD370D5783900C6F0503C387372FBFF44" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{76EFBC58-797F-42F1-AE22-74AA368945FA}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="11_2B59D2BFD370D5783900C6F0503C387372FBFF44" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F814381-CE92-461A-9C66-86D2B171CAD6}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="1080" yWindow="1080" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$C$1:$C$7</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -743,6 +746,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="C1:C7" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>